<commit_message>
feat: export complete student records
</commit_message>
<xml_diff>
--- a/public/Ficha_Alumno_TEMPLATE.xlsx
+++ b/public/Ficha_Alumno_TEMPLATE.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="63">
   <si>
     <t>FICHA DE INSCRIPCIÓN Y DATOS DEL ALUMNO</t>
   </si>
@@ -88,6 +88,9 @@
     <t>Última regeneración:</t>
   </si>
   <si>
+    <t>Grado:</t>
+  </si>
+  <si>
     <t>4. AUTORIZACIONES DE RETIRO</t>
   </si>
   <si>
@@ -140,6 +143,66 @@
   </si>
   <si>
     <t>Psicopedagogo:</t>
+  </si>
+  <si>
+    <t>7. INFORMACIÓN ADICIONAL</t>
+  </si>
+  <si>
+    <t>Autenticación en dos pasos:</t>
+  </si>
+  <si>
+    <t>Función:</t>
+  </si>
+  <si>
+    <t>Última vez:</t>
+  </si>
+  <si>
+    <t>Firma Digital:</t>
+  </si>
+  <si>
+    <t>Piso:</t>
+  </si>
+  <si>
+    <t>Departamento:</t>
+  </si>
+  <si>
+    <t>Torre:</t>
+  </si>
+  <si>
+    <t>Legajo:</t>
+  </si>
+  <si>
+    <t>Libro Matriz:</t>
+  </si>
+  <si>
+    <t>Folio:</t>
+  </si>
+  <si>
+    <t>Conducta:</t>
+  </si>
+  <si>
+    <t>Colegio de procedencia:</t>
+  </si>
+  <si>
+    <t>Tutor principal:</t>
+  </si>
+  <si>
+    <t>Tratamiento Impositivo:</t>
+  </si>
+  <si>
+    <t>CUIT:</t>
+  </si>
+  <si>
+    <t>8. LEGAJO</t>
+  </si>
+  <si>
+    <t>Cita Preinscripción:</t>
+  </si>
+  <si>
+    <t>Admisión:</t>
+  </si>
+  <si>
+    <t>Escuela Anterior:</t>
   </si>
 </sst>
 </file>
@@ -540,7 +603,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D34"/>
+  <dimension ref="A1:D50"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="9.140625"/>
   <cols>
     <col min="1" max="1" width="25" customWidth="1"/>
@@ -687,9 +750,17 @@
       </c>
       <c r="D18" s="4"/>
     </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A19" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B19" s="4"/>
+      <c r="C19" s="4"/>
+      <c r="D19" s="4"/>
+    </row>
     <row r="20" ht="24" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B20"/>
       <c r="C20"/>
@@ -697,27 +768,27 @@
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B21" s="4"/>
       <c r="C21" s="3" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D21" s="4"/>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B22" s="4"/>
       <c r="C22" s="3" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D22" s="4"/>
     </row>
     <row r="24" ht="24" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B24"/>
       <c r="C24"/>
@@ -725,7 +796,7 @@
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B25" s="4"/>
       <c r="C25" s="5"/>
@@ -733,7 +804,7 @@
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" s="3" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B26" s="4"/>
       <c r="C26" s="5"/>
@@ -741,7 +812,7 @@
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B27" s="4"/>
       <c r="C27" s="5"/>
@@ -749,7 +820,7 @@
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" s="3" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B28" s="4"/>
       <c r="C28" s="5"/>
@@ -757,7 +828,7 @@
     </row>
     <row r="30" ht="24" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B30"/>
       <c r="C30"/>
@@ -765,52 +836,177 @@
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B31" s="4"/>
       <c r="C31" s="3" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D31" s="4"/>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" s="3" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B32" s="4"/>
       <c r="C32" s="3" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D32" s="4"/>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" s="3" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B33" s="4"/>
       <c r="C33" s="3" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D33" s="4"/>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34" s="3" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B34" s="4"/>
       <c r="C34" s="3" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D34" s="4"/>
     </row>
+    <row r="36" ht="24" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A36" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B36"/>
+      <c r="C36"/>
+      <c r="D36"/>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A37" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="B37" s="4"/>
+      <c r="C37" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="D37" s="4"/>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A38" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="B38" s="4"/>
+      <c r="C38" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="D38" s="4"/>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A39" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="B39" s="4"/>
+      <c r="C39" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="D39" s="4"/>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A40" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="B40" s="4"/>
+      <c r="C40" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="D40" s="4"/>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A41" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="B41" s="4"/>
+      <c r="C41" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="D41" s="4"/>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A42" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="B42" s="4"/>
+      <c r="C42" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="D42" s="4"/>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A43" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="B43" s="4"/>
+      <c r="C43" s="4"/>
+      <c r="D43" s="4"/>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A44" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="B44" s="4"/>
+      <c r="C44" s="4"/>
+      <c r="D44" s="4"/>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A45" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="B45" s="4"/>
+      <c r="C45" s="4"/>
+      <c r="D45" s="4"/>
+    </row>
+    <row r="47" ht="24" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A47" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B47"/>
+      <c r="C47"/>
+      <c r="D47"/>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A48" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="B48" s="4"/>
+      <c r="C48" s="4"/>
+      <c r="D48" s="4"/>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A49" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="B49" s="4"/>
+      <c r="C49" s="4"/>
+      <c r="D49" s="4"/>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A50" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="B50" s="4"/>
+      <c r="C50" s="4"/>
+      <c r="D50" s="4"/>
+    </row>
   </sheetData>
-  <mergeCells count="13">
+  <mergeCells count="22">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A3:D3"/>
     <mergeCell ref="B4:D4"/>
     <mergeCell ref="A11:D11"/>
     <mergeCell ref="B12:D12"/>
     <mergeCell ref="A16:D16"/>
+    <mergeCell ref="B19:D19"/>
     <mergeCell ref="A20:D20"/>
     <mergeCell ref="A24:D24"/>
     <mergeCell ref="B25:D25"/>
@@ -818,6 +1014,14 @@
     <mergeCell ref="B27:D27"/>
     <mergeCell ref="B28:D28"/>
     <mergeCell ref="A30:D30"/>
+    <mergeCell ref="A36:D36"/>
+    <mergeCell ref="B43:D43"/>
+    <mergeCell ref="B44:D44"/>
+    <mergeCell ref="B45:D45"/>
+    <mergeCell ref="A47:D47"/>
+    <mergeCell ref="B48:D48"/>
+    <mergeCell ref="B49:D49"/>
+    <mergeCell ref="B50:D50"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>